<commit_message>
Separar equipe de processo: remover nomes fixos do script e planilha, criar equipe-atual.md
</commit_message>
<xml_diff>
--- a/planilha-acompanhamento-leads.xlsx
+++ b/planilha-acompanhamento-leads.xlsx
@@ -518,7 +518,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Legenda: preencha apenas as células com fundo amarelo. As colunas com lista suspensa (curso, SDR, status etc.) usam os valores da aba "Listas (validação)" — não digite valores fora da lista. Linha 5 é um exemplo preenchido; apague-a ou substitua pelos dados reais antes do uso.</t>
+          <t>Legenda: preencha apenas as células com fundo amarelo. As colunas com lista suspensa (curso, SDR, status etc.) usam os valores da aba "Listas (validação)" — não digite valores fora da lista. Linha 5 é um exemplo preenchido; apague-a ou substitua pelos dados reais antes do uso. Os nomes de SDR e Seller na aba de validação mudam conforme a equipe atual (ver equipe-atual.md) — edite apenas essa lista quando alguém entrar ou sair, sem mexer no resto da planilha.</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2328,7 @@
       <formula1>'Listas (validação)'!$A$2:$A$4</formula1>
     </dataValidation>
     <dataValidation sqref="F5:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Selecione um valor da lista." type="list">
-      <formula1>'Listas (validação)'!$B$2:$B$4</formula1>
+      <formula1>'Listas (validação)'!$B$2:$B$5</formula1>
     </dataValidation>
     <dataValidation sqref="K5:K60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Selecione um valor da lista." type="list">
       <formula1>'Listas (validação)'!$C$2:$C$4</formula1>
@@ -2349,7 +2349,7 @@
       <formula1>'Listas (validação)'!$C$2:$C$4</formula1>
     </dataValidation>
     <dataValidation sqref="T5:T60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Selecione um valor da lista." type="list">
-      <formula1>'Listas (validação)'!$D$2:$D$2</formula1>
+      <formula1>'Listas (validação)'!$D$2:$D$5</formula1>
     </dataValidation>
     <dataValidation sqref="U5:U60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Selecione um valor da lista." type="list">
       <formula1>'Listas (validação)'!$E$2:$E$9</formula1>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Giovanna</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Nadja</t>
+          <t>Carla</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -2451,12 +2451,17 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Sadah</t>
+          <t>Geovanna</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Não</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Nadja</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -2478,26 +2483,41 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
+          <t>Sarah</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Vania</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Matriculou</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Não atendeu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="7" t="inlineStr">
+        <is>
           <t>Henzo</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Matriculou</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Não atendeu</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Kaique</t>
+        </is>
+      </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Não matriculou</t>
@@ -2651,7 +2671,7 @@
     <row r="23">
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Encaminhado para Nadja</t>
+          <t>Encaminhado para a Seller</t>
         </is>
       </c>
     </row>

</xml_diff>